<commit_message>
Add metadata model, impact analysis, glossary, and data dictionary
</commit_message>
<xml_diff>
--- a/04_metadata_and_lineage/business-glossary.xlsx
+++ b/04_metadata_and_lineage/business-glossary.xlsx
@@ -8,15 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\enterprise-data-governance-operating-system\04_metadata_and_lineage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8EB444B4-CAEA-4114-800B-BB20F782C7AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{300B0758-9324-4668-8C99-A321ED4F87BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{5B0C5EF1-E731-4DE9-9191-DAFD0A768F15}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="1" xr2:uid="{5B0C5EF1-E731-4DE9-9191-DAFD0A768F15}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="Glossary" sheetId="2" r:id="rId2"/>
     <sheet name="Domains" sheetId="1" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Domains!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Glossary!$A$1:$N$6</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,11 +42,296 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="88">
+  <si>
+    <t>Business Glossary Workbook</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Provides a structured register of approved business terms, definitions, owners, stewards, and review dates.</t>
+  </si>
+  <si>
+    <t>How to use</t>
+  </si>
+  <si>
+    <t>Add one row per approved or candidate term. Use this workbook to reduce definition drift across reports, dashboards, and operational workflows.</t>
+  </si>
+  <si>
+    <t>Governance rule</t>
+  </si>
+  <si>
+    <t>Approved terms should have a named owner, clear definition, domain, and review date.</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Example Assets</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>Customer and client master data and identifiers</t>
+  </si>
+  <si>
+    <t>customer_master, customer_profile</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>Operational service delivery, work activity, and workflow data</t>
+  </si>
+  <si>
+    <t>service_request, work_order</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Financial transactions, balances, and reporting data</t>
+  </si>
+  <si>
+    <t>transaction_fact, finance_dashboard</t>
+  </si>
+  <si>
+    <t>Asset</t>
+  </si>
+  <si>
+    <t>Physical asset, infrastructure, and asset lifecycle data</t>
+  </si>
+  <si>
+    <t>asset_register, asset_component</t>
+  </si>
+  <si>
+    <t>Reporting</t>
+  </si>
+  <si>
+    <t>Certified shared reporting outputs and KPI assets</t>
+  </si>
+  <si>
+    <t>executive_dashboard, management_scorecard</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>Controlled lists, code values, and supporting reference data</t>
+  </si>
+  <si>
+    <t>status_codes, geography_reference</t>
+  </si>
+  <si>
+    <t>Term ID</t>
+  </si>
+  <si>
+    <t>Term Name</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Steward</t>
+  </si>
+  <si>
+    <t>Synonyms</t>
+  </si>
+  <si>
+    <t>Non-Approved Terms</t>
+  </si>
+  <si>
+    <t>Calculation Rule</t>
+  </si>
+  <si>
+    <t>Source Reference</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Effective Date</t>
+  </si>
+  <si>
+    <t>Review Date</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>TERM-001</t>
+  </si>
+  <si>
+    <t>Active Customer</t>
+  </si>
+  <si>
+    <t>A customer with at least one qualifying interaction or transaction in the approved review period.</t>
+  </si>
+  <si>
+    <t>Head of Customer Data</t>
+  </si>
+  <si>
+    <t>Customer Data Steward</t>
+  </si>
+  <si>
+    <t>Current Customer</t>
+  </si>
+  <si>
+    <t>Live Customer Count</t>
+  </si>
+  <si>
+    <t>Count distinct customer_id where qualifying_activity_flag = Y</t>
+  </si>
+  <si>
+    <t>Customer KPI Standard</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Align across shared reporting</t>
+  </si>
+  <si>
+    <t>TERM-002</t>
+  </si>
+  <si>
+    <t>Service Request</t>
+  </si>
+  <si>
+    <t>A formal request logged for operational action, inspection, service delivery, or follow-up.</t>
+  </si>
+  <si>
+    <t>Operations Manager</t>
+  </si>
+  <si>
+    <t>Operations Data Steward</t>
+  </si>
+  <si>
+    <t>Case, Ticket</t>
+  </si>
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Operations SOP</t>
+  </si>
+  <si>
+    <t>Used across intake and reporting</t>
+  </si>
+  <si>
+    <t>TERM-003</t>
+  </si>
+  <si>
+    <t>Critical Data Element</t>
+  </si>
+  <si>
+    <t>A field or attribute whose failure would materially affect reporting, operations, compliance, or access decisions.</t>
+  </si>
+  <si>
+    <t>Governance Lead</t>
+  </si>
+  <si>
+    <t>Reporting Steward</t>
+  </si>
+  <si>
+    <t>CDE</t>
+  </si>
+  <si>
+    <t>DQ Framework</t>
+  </si>
+  <si>
+    <t>Used in control design</t>
+  </si>
+  <si>
+    <t>TERM-004</t>
+  </si>
+  <si>
+    <t>Certified Report</t>
+  </si>
+  <si>
+    <t>A reporting output that has completed the required review and control steps for intended business use.</t>
+  </si>
+  <si>
+    <t>Reporting Director</t>
+  </si>
+  <si>
+    <t>Validated Report</t>
+  </si>
+  <si>
+    <t>Published File</t>
+  </si>
+  <si>
+    <t>Must complete required controls and sign-off</t>
+  </si>
+  <si>
+    <t>Reporting Certification Procedure</t>
+  </si>
+  <si>
+    <t>Important for release discipline</t>
+  </si>
+  <si>
+    <t>TERM-005</t>
+  </si>
+  <si>
+    <t>Sensitive Data</t>
+  </si>
+  <si>
+    <t>Data requiring elevated handling due to privacy, confidentiality, legal, or operational risk.</t>
+  </si>
+  <si>
+    <t>Privacy Lead</t>
+  </si>
+  <si>
+    <t>Governance Steward</t>
+  </si>
+  <si>
+    <t>Restricted Data</t>
+  </si>
+  <si>
+    <t>Private-ish Data</t>
+  </si>
+  <si>
+    <t>Classification Model</t>
+  </si>
+  <si>
+    <t>Link to access controls</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +358,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,27 +677,425 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CFEF63A-8463-4CE7-9C93-178D758B4DBD}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="30.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="117.265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="135" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86210F69-9BC8-40F1-94C0-F22C60E08D38}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="89.53125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.3984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.19921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.73046875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.59765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="49.46484375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.1328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" t="s">
+        <v>50</v>
+      </c>
+      <c r="L2" s="3">
+        <v>46023</v>
+      </c>
+      <c r="M2" s="3">
+        <v>46204</v>
+      </c>
+      <c r="N2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="3">
+        <v>46023</v>
+      </c>
+      <c r="M3" s="3">
+        <v>46204</v>
+      </c>
+      <c r="N3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K4" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="3">
+        <v>46023</v>
+      </c>
+      <c r="M4" s="3">
+        <v>46204</v>
+      </c>
+      <c r="N4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" s="3">
+        <v>46023</v>
+      </c>
+      <c r="M5" s="3">
+        <v>46204</v>
+      </c>
+      <c r="N5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" t="s">
+        <v>85</v>
+      </c>
+      <c r="I6" t="s">
+        <v>59</v>
+      </c>
+      <c r="J6" t="s">
+        <v>86</v>
+      </c>
+      <c r="K6" t="s">
+        <v>50</v>
+      </c>
+      <c r="L6" s="3">
+        <v>46023</v>
+      </c>
+      <c r="M6" s="3">
+        <v>46204</v>
+      </c>
+      <c r="N6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N6" xr:uid="{86210F69-9BC8-40F1-94C0-F22C60E08D38}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C12C385E-7777-4633-B0B6-FEB3D1CF9167}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C7" xr:uid="{C12C385E-7777-4633-B0B6-FEB3D1CF9167}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>